<commit_message>
Probando la aplicacion 28-04-2026
</commit_message>
<xml_diff>
--- a/Excel/CIRCUITO ISSUNNE/Planilla_Seguimiento_UPCM_ISSUNNE.xlsx
+++ b/Excel/CIRCUITO ISSUNNE/Planilla_Seguimiento_UPCM_ISSUNNE.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Hernán\Desktop\CIRCUITO ISSUNNE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Hernán\Desktop\Administracion HernanMayol\Python_ISSUNNE\Excel\CIRCUITO ISSUNNE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99847F7F-26F2-42F2-96A5-0B4DBABF17B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FFB6F35-0B89-48A9-86B6-12C826873641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1036,23 +1036,23 @@
       <c r="B3" s="12"/>
       <c r="C3" s="12"/>
       <c r="D3" s="5">
-        <v>46019</v>
+        <v>46133</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="5">
-        <v>46024</v>
+        <v>46133</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="12" t="s">
         <v>14</v>
       </c>
       <c r="I3" s="5">
-        <v>46024</v>
+        <v>46134</v>
       </c>
       <c r="J3" s="9"/>
       <c r="K3" s="6">
         <f t="shared" ca="1" si="0"/>
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="L3" s="14" t="s">
         <v>14</v>
@@ -1065,7 +1065,7 @@
       )
    )
 )</f>
-        <v>🔴 Pendiente</v>
+        <v>🟠 Pendiente</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -1073,11 +1073,11 @@
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="7">
-        <v>46047</v>
+        <v>46117</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" s="7">
-        <v>46049</v>
+        <v>46118</v>
       </c>
       <c r="G4" s="7"/>
       <c r="H4" s="13" t="s">
@@ -1087,7 +1087,7 @@
       <c r="J4" s="10"/>
       <c r="K4" s="8">
         <f t="shared" ca="1" si="0"/>
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="L4" s="14" t="s">
         <v>14</v>
@@ -1100,7 +1100,7 @@
       )
    )
 )</f>
-        <v>🟠 Pendiente</v>
+        <v>🔴 Pendiente</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -1169,7 +1169,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
   <tableParts count="1">
     <tablePart r:id="rId2"/>
   </tableParts>

</xml_diff>